<commit_message>
doc: convert all excel file to english
</commit_message>
<xml_diff>
--- a/Tests/excel/module01_test_cases.xlsx
+++ b/Tests/excel/module01_test_cases.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Module01" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Report" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Module01" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Module01'!$A$1:$N$40</definedName>
@@ -398,14 +398,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -429,10 +429,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="FF0000"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -456,10 +456,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="FFFF00"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -483,10 +483,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="00FF00"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -515,8 +515,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -542,8 +542,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -569,7 +569,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>7</col>
@@ -584,9 +584,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>

</xml_diff>

<commit_message>
doc: completed testing for module 2
</commit_message>
<xml_diff>
--- a/Tests/excel/module01_test_cases.xlsx
+++ b/Tests/excel/module01_test_cases.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Module01" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Module01'!$A$1:$N$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Module01'!$A$1:$O$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1003,15 +1003,15 @@
         </is>
       </c>
       <c r="C9" s="24">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A9, 'Module01'!$M$2:$M$34, "High")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A9, 'Module01'!$N$2:$N$34, "High")</f>
         <v/>
       </c>
       <c r="D9" s="25">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A9, 'Module01'!$M$2:$M$34, "Medium")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A9, 'Module01'!$N$2:$N$34, "Medium")</f>
         <v/>
       </c>
       <c r="E9" s="26">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A9, 'Module01'!$M$2:$M$34, "Low")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A9, 'Module01'!$N$2:$N$34, "Low")</f>
         <v/>
       </c>
       <c r="F9" s="27">
@@ -1031,15 +1031,15 @@
         </is>
       </c>
       <c r="C10" s="30">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A10, 'Module01'!$M$2:$M$34, "High")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A10, 'Module01'!$N$2:$N$34, "High")</f>
         <v/>
       </c>
       <c r="D10" s="31">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A10, 'Module01'!$M$2:$M$34, "Medium")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A10, 'Module01'!$N$2:$N$34, "Medium")</f>
         <v/>
       </c>
       <c r="E10" s="32">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A10, 'Module01'!$M$2:$M$34, "Low")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A10, 'Module01'!$N$2:$N$34, "Low")</f>
         <v/>
       </c>
       <c r="F10" s="33">
@@ -1059,15 +1059,15 @@
         </is>
       </c>
       <c r="C11" s="24">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A11, 'Module01'!$M$2:$M$34, "High")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A11, 'Module01'!$N$2:$N$34, "High")</f>
         <v/>
       </c>
       <c r="D11" s="25">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A11, 'Module01'!$M$2:$M$34, "Medium")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A11, 'Module01'!$N$2:$N$34, "Medium")</f>
         <v/>
       </c>
       <c r="E11" s="26">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A11, 'Module01'!$M$2:$M$34, "Low")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A11, 'Module01'!$N$2:$N$34, "Low")</f>
         <v/>
       </c>
       <c r="F11" s="27">
@@ -1087,15 +1087,15 @@
         </is>
       </c>
       <c r="C12" s="30">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A12, 'Module01'!$M$2:$M$34, "High")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A12, 'Module01'!$N$2:$N$34, "High")</f>
         <v/>
       </c>
       <c r="D12" s="31">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A12, 'Module01'!$M$2:$M$34, "Medium")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A12, 'Module01'!$N$2:$N$34, "Medium")</f>
         <v/>
       </c>
       <c r="E12" s="32">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A12, 'Module01'!$M$2:$M$34, "Low")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A12, 'Module01'!$N$2:$N$34, "Low")</f>
         <v/>
       </c>
       <c r="F12" s="33">
@@ -1115,15 +1115,15 @@
         </is>
       </c>
       <c r="C13" s="24">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A13, 'Module01'!$M$2:$M$34, "High")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A13, 'Module01'!$N$2:$N$34, "High")</f>
         <v/>
       </c>
       <c r="D13" s="25">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A13, 'Module01'!$M$2:$M$34, "Medium")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A13, 'Module01'!$N$2:$N$34, "Medium")</f>
         <v/>
       </c>
       <c r="E13" s="26">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A13, 'Module01'!$M$2:$M$34, "Low")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A13, 'Module01'!$N$2:$N$34, "Low")</f>
         <v/>
       </c>
       <c r="F13" s="27">
@@ -1143,15 +1143,15 @@
         </is>
       </c>
       <c r="C14" s="30">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A14, 'Module01'!$M$2:$M$34, "High")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A14, 'Module01'!$N$2:$N$34, "High")</f>
         <v/>
       </c>
       <c r="D14" s="31">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A14, 'Module01'!$M$2:$M$34, "Medium")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A14, 'Module01'!$N$2:$N$34, "Medium")</f>
         <v/>
       </c>
       <c r="E14" s="32">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A14, 'Module01'!$M$2:$M$34, "Low")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A14, 'Module01'!$N$2:$N$34, "Low")</f>
         <v/>
       </c>
       <c r="F14" s="33">
@@ -1171,15 +1171,15 @@
         </is>
       </c>
       <c r="C15" s="24">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A15, 'Module01'!$M$2:$M$34, "High")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A15, 'Module01'!$N$2:$N$34, "High")</f>
         <v/>
       </c>
       <c r="D15" s="25">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A15, 'Module01'!$M$2:$M$34, "Medium")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A15, 'Module01'!$N$2:$N$34, "Medium")</f>
         <v/>
       </c>
       <c r="E15" s="26">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A15, 'Module01'!$M$2:$M$34, "Low")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A15, 'Module01'!$N$2:$N$34, "Low")</f>
         <v/>
       </c>
       <c r="F15" s="27">
@@ -1199,15 +1199,15 @@
         </is>
       </c>
       <c r="C16" s="30">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A16, 'Module01'!$M$2:$M$34, "High")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A16, 'Module01'!$N$2:$N$34, "High")</f>
         <v/>
       </c>
       <c r="D16" s="31">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A16, 'Module01'!$M$2:$M$34, "Medium")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A16, 'Module01'!$N$2:$N$34, "Medium")</f>
         <v/>
       </c>
       <c r="E16" s="32">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A16, 'Module01'!$M$2:$M$34, "Low")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A16, 'Module01'!$N$2:$N$34, "Low")</f>
         <v/>
       </c>
       <c r="F16" s="33">
@@ -1227,15 +1227,15 @@
         </is>
       </c>
       <c r="C17" s="24">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A17, 'Module01'!$M$2:$M$34, "High")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A17, 'Module01'!$N$2:$N$34, "High")</f>
         <v/>
       </c>
       <c r="D17" s="25">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A17, 'Module01'!$M$2:$M$34, "Medium")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A17, 'Module01'!$N$2:$N$34, "Medium")</f>
         <v/>
       </c>
       <c r="E17" s="26">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A17, 'Module01'!$M$2:$M$34, "Low")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A17, 'Module01'!$N$2:$N$34, "Low")</f>
         <v/>
       </c>
       <c r="F17" s="27">
@@ -1255,15 +1255,15 @@
         </is>
       </c>
       <c r="C18" s="30">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A18, 'Module01'!$M$2:$M$34, "High")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A18, 'Module01'!$N$2:$N$34, "High")</f>
         <v/>
       </c>
       <c r="D18" s="31">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A18, 'Module01'!$M$2:$M$34, "Medium")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A18, 'Module01'!$N$2:$N$34, "Medium")</f>
         <v/>
       </c>
       <c r="E18" s="32">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A18, 'Module01'!$M$2:$M$34, "Low")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A18, 'Module01'!$N$2:$N$34, "Low")</f>
         <v/>
       </c>
       <c r="F18" s="33">
@@ -1283,15 +1283,15 @@
         </is>
       </c>
       <c r="C19" s="24">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A19, 'Module01'!$M$2:$M$34, "High")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A19, 'Module01'!$N$2:$N$34, "High")</f>
         <v/>
       </c>
       <c r="D19" s="25">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A19, 'Module01'!$M$2:$M$34, "Medium")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A19, 'Module01'!$N$2:$N$34, "Medium")</f>
         <v/>
       </c>
       <c r="E19" s="26">
-        <f>COUNTIFS('Module01'!$C$2:$C$34, A19, 'Module01'!$M$2:$M$34, "Low")</f>
+        <f>COUNTIFS('Module01'!$C$2:$C$34, A19, 'Module01'!$N$2:$N$34, "Low")</f>
         <v/>
       </c>
       <c r="F19" s="27">
@@ -1338,7 +1338,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N34"/>
+  <dimension ref="A1:O34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1353,8 +1353,9 @@
     <col width="48" customWidth="1" min="10" max="10"/>
     <col width="36" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="32" customWidth="1" min="14" max="14"/>
+    <col width="25" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="32" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -1420,10 +1421,15 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -1494,12 +1500,13 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="M2" s="6" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N2" s="4" t="inlineStr">
+      <c r="O2" s="4" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F01, Scenario: BS-01</t>
         </is>
@@ -1569,12 +1576,13 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="M3" s="6" t="inlineStr">
+      <c r="M3" s="7" t="inlineStr"/>
+      <c r="N3" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N3" s="9" t="inlineStr">
+      <c r="O3" s="9" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F01, Scenario: BS-01</t>
         </is>
@@ -1644,12 +1652,13 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="M4" s="6" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr"/>
+      <c r="N4" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N4" s="4" t="inlineStr">
+      <c r="O4" s="4" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F01, Scenario: BS-01</t>
         </is>
@@ -1719,12 +1728,13 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="M5" s="6" t="inlineStr">
+      <c r="M5" s="7" t="inlineStr"/>
+      <c r="N5" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N5" s="9" t="inlineStr">
+      <c r="O5" s="9" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F01, Scenario: BS-01</t>
         </is>
@@ -1794,12 +1804,13 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="M6" s="6" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr"/>
+      <c r="N6" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N6" s="4" t="inlineStr">
+      <c r="O6" s="4" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F01, Scenario: BS-01</t>
         </is>
@@ -1869,12 +1880,13 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="M7" s="6" t="inlineStr">
+      <c r="M7" s="7" t="inlineStr"/>
+      <c r="N7" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N7" s="9" t="inlineStr">
+      <c r="O7" s="9" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F01, Scenario: BS-01</t>
         </is>
@@ -1944,12 +1956,13 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="M8" s="6" t="inlineStr">
+      <c r="M8" s="2" t="inlineStr"/>
+      <c r="N8" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N8" s="4" t="inlineStr">
+      <c r="O8" s="4" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F01, Scenario: BS-01</t>
         </is>
@@ -2019,12 +2032,13 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="M9" s="6" t="inlineStr">
+      <c r="M9" s="7" t="inlineStr"/>
+      <c r="N9" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N9" s="9" t="inlineStr">
+      <c r="O9" s="9" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F02, Scenario: BS-02</t>
         </is>
@@ -2094,12 +2108,13 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="M10" s="6" t="inlineStr">
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N10" s="4" t="inlineStr">
+      <c r="O10" s="4" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F02, Scenario: BS-02</t>
         </is>
@@ -2169,12 +2184,13 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="M11" s="6" t="inlineStr">
+      <c r="M11" s="7" t="inlineStr"/>
+      <c r="N11" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N11" s="9" t="inlineStr">
+      <c r="O11" s="9" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F02, Scenario: BS-02</t>
         </is>
@@ -2243,12 +2259,13 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="M12" s="6" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N12" s="4" t="inlineStr">
+      <c r="O12" s="4" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F03, Scenario: BS-03</t>
         </is>
@@ -2318,12 +2335,13 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="M13" s="6" t="inlineStr">
+      <c r="M13" s="7" t="inlineStr"/>
+      <c r="N13" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N13" s="9" t="inlineStr">
+      <c r="O13" s="9" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F03, Scenario: BS-03</t>
         </is>
@@ -2392,12 +2410,13 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="M14" s="10" t="inlineStr">
+      <c r="M14" s="2" t="inlineStr"/>
+      <c r="N14" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="N14" s="4" t="inlineStr">
+      <c r="O14" s="4" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F03, Scenario: BS-03</t>
         </is>
@@ -2470,12 +2489,13 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="M15" s="6" t="inlineStr">
+      <c r="M15" s="7" t="inlineStr"/>
+      <c r="N15" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N15" s="9" t="inlineStr">
+      <c r="O15" s="9" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F04, Scenario: BS-04</t>
         </is>
@@ -2546,12 +2566,13 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="M16" s="6" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr"/>
+      <c r="N16" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N16" s="4" t="inlineStr">
+      <c r="O16" s="4" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F04, Scenario: BS-04</t>
         </is>
@@ -2621,12 +2642,13 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="M17" s="6" t="inlineStr">
+      <c r="M17" s="7" t="inlineStr"/>
+      <c r="N17" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N17" s="9" t="inlineStr">
+      <c r="O17" s="9" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F04, Scenario: BS-04</t>
         </is>
@@ -2695,12 +2717,13 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="M18" s="6" t="inlineStr">
+      <c r="M18" s="2" t="inlineStr"/>
+      <c r="N18" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N18" s="4" t="inlineStr">
+      <c r="O18" s="4" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F05, Scenario: BS-05</t>
         </is>
@@ -2769,12 +2792,13 @@
           <t>Failed</t>
         </is>
       </c>
-      <c r="M19" s="6" t="inlineStr">
+      <c r="M19" s="7" t="inlineStr"/>
+      <c r="N19" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N19" s="9" t="inlineStr">
+      <c r="O19" s="9" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F05, Scenario: BS-05</t>
         </is>
@@ -2843,12 +2867,13 @@
           <t>Failed</t>
         </is>
       </c>
-      <c r="M20" s="6" t="inlineStr">
+      <c r="M20" s="2" t="inlineStr"/>
+      <c r="N20" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N20" s="4" t="inlineStr">
+      <c r="O20" s="4" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F05, Scenario: BS-05</t>
         </is>
@@ -2918,12 +2943,13 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="M21" s="6" t="inlineStr">
+      <c r="M21" s="7" t="inlineStr"/>
+      <c r="N21" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N21" s="9" t="inlineStr">
+      <c r="O21" s="9" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F06, Scenario: BS-06</t>
         </is>
@@ -2993,12 +3019,13 @@
           <t>Failed</t>
         </is>
       </c>
-      <c r="M22" s="6" t="inlineStr">
+      <c r="M22" s="2" t="inlineStr"/>
+      <c r="N22" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N22" s="4" t="inlineStr">
+      <c r="O22" s="4" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F07, Scenario: BS-07</t>
         </is>
@@ -3068,12 +3095,13 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="M23" s="6" t="inlineStr">
+      <c r="M23" s="7" t="inlineStr"/>
+      <c r="N23" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N23" s="9" t="inlineStr">
+      <c r="O23" s="9" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F08, Scenario: BS-08</t>
         </is>
@@ -3143,12 +3171,13 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="M24" s="6" t="inlineStr">
+      <c r="M24" s="2" t="inlineStr"/>
+      <c r="N24" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N24" s="4" t="inlineStr">
+      <c r="O24" s="4" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F08, Scenario: BS-08</t>
         </is>
@@ -3217,12 +3246,13 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="M25" s="10" t="inlineStr">
+      <c r="M25" s="7" t="inlineStr"/>
+      <c r="N25" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="N25" s="9" t="inlineStr">
+      <c r="O25" s="9" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F09, Scenario: BS-09</t>
         </is>
@@ -3292,12 +3322,13 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="M26" s="10" t="inlineStr">
+      <c r="M26" s="2" t="inlineStr"/>
+      <c r="N26" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="N26" s="4" t="inlineStr">
+      <c r="O26" s="4" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F09, Scenario: BS-10</t>
         </is>
@@ -3365,12 +3396,13 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="M27" s="10" t="inlineStr">
+      <c r="M27" s="7" t="inlineStr"/>
+      <c r="N27" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="N27" s="9" t="inlineStr">
+      <c r="O27" s="9" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F10, Scenario: BS-11</t>
         </is>
@@ -3439,12 +3471,13 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="M28" s="10" t="inlineStr">
+      <c r="M28" s="2" t="inlineStr"/>
+      <c r="N28" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="N28" s="4" t="inlineStr">
+      <c r="O28" s="4" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F10, Scenario: BS-11</t>
         </is>
@@ -3512,12 +3545,13 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="M29" s="6" t="inlineStr">
+      <c r="M29" s="7" t="inlineStr"/>
+      <c r="N29" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N29" s="9" t="inlineStr">
+      <c r="O29" s="9" t="inlineStr">
         <is>
           <t>Related Requirement: General Business Rules, Scenario: BS-12</t>
         </is>
@@ -3585,12 +3619,13 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="M30" s="6" t="inlineStr">
+      <c r="M30" s="2" t="inlineStr"/>
+      <c r="N30" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N30" s="4" t="inlineStr">
+      <c r="O30" s="4" t="inlineStr">
         <is>
           <t>Related Requirement: General Business Rules, Scenario: BS-12</t>
         </is>
@@ -3659,12 +3694,13 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="M31" s="6" t="inlineStr">
+      <c r="M31" s="7" t="inlineStr"/>
+      <c r="N31" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N31" s="9" t="inlineStr">
+      <c r="O31" s="9" t="inlineStr">
         <is>
           <t>Related Requirement: General Business Rules, Authorization</t>
         </is>
@@ -3733,12 +3769,13 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="M32" s="6" t="inlineStr">
+      <c r="M32" s="2" t="inlineStr"/>
+      <c r="N32" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N32" s="4" t="inlineStr">
+      <c r="O32" s="4" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F05, Validation Rules</t>
         </is>
@@ -3807,12 +3844,13 @@
           <t>Passed</t>
         </is>
       </c>
-      <c r="M33" s="10" t="inlineStr">
+      <c r="M33" s="7" t="inlineStr"/>
+      <c r="N33" s="10" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="N33" s="9" t="inlineStr">
+      <c r="O33" s="9" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F09, Search &amp; Filter</t>
         </is>
@@ -3882,24 +3920,25 @@
           <t>Failed</t>
         </is>
       </c>
-      <c r="M34" s="6" t="inlineStr">
+      <c r="M34" s="2" t="inlineStr"/>
+      <c r="N34" s="6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N34" s="4" t="inlineStr">
+      <c r="O34" s="4" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F06, Validation Rules</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N34"/>
+  <autoFilter ref="A1:O34"/>
   <dataValidations count="2">
     <dataValidation sqref="L2:L134" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Status" error="Please select a valid state: Passed, Failed, or Not Run" type="list">
       <formula1>"Passed,Failed,Not Run"</formula1>
     </dataValidation>
-    <dataValidation sqref="M2:M134" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Priority" error="Please select a valid priority: High, Medium, or Low" type="list">
+    <dataValidation sqref="N2:N134" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Priority" error="Please select a valid priority: High, Medium, or Low" type="list">
       <formula1>"High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>